<commit_message>
Corrige semáforo de Entregas Próximas (colores consistentes)
- Quita la banda cebra y sube la prioridad del semáforo (21-24) por
  encima del borde, de modo que el color de estado SIEMPRE se aplique.
- Antes la banda (prioridad mayor) tapaba el color en las filas pares:
  'Próximo a vencer' se veía resaltado una fila sí y otra no, y las
  tareas al 100% no quedaban en verde. Ahora cada estado colorea de
  forma uniforme en todas las filas (incl. Completado en verde).

https://claude.ai/code/session_01T2X5Sdkmy5GoJRwojb8uhJ
</commit_message>
<xml_diff>
--- a/Diagrama_de_Gantt___Proyecto_Datos_Op._Complejas_080626.xlsx
+++ b/Diagrama_de_Gantt___Proyecto_Datos_Op._Complejas_080626.xlsx
@@ -21112,26 +21112,23 @@
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="B5:I5"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:I156">
-    <cfRule type="expression" dxfId="22" priority="31">
-      <formula>AND($D7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+  <conditionalFormatting sqref="G7:H156">
+    <cfRule type="expression" dxfId="23" priority="21">
+      <formula>$G7="Vencido"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="32">
-      <formula>$D7&lt;&gt;""</formula>
+    <cfRule type="expression" dxfId="24" priority="22">
+      <formula>$G7="Próximo a vencer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="23">
+      <formula>$G7="En curso"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="24">
+      <formula>$G7="Completado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G7:H156">
-    <cfRule type="expression" dxfId="23" priority="33">
-      <formula>$G7="Vencido"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="34">
-      <formula>$G7="Próximo a vencer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="25" priority="35">
-      <formula>$G7="En curso"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="26" priority="36">
-      <formula>$G7="Completado"</formula>
+  <conditionalFormatting sqref="B7:I156">
+    <cfRule type="expression" dxfId="21" priority="40">
+      <formula>$D7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>